<commit_message>
br1: plotted average max and average min errors
</commit_message>
<xml_diff>
--- a/results/no_constraints/256nodes_diameter79_cutoff1.0-repetitions10-overlap100.xlsx
+++ b/results/no_constraints/256nodes_diameter79_cutoff1.0-repetitions10-overlap100.xlsx
@@ -1,16 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ksuprod-my.sharepoint.com/personal/sbhatt23_kent_edu/Documents/Desktop/Distributed Directories Under Predictions/results/no_constraints/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_2900FD3EECB7D80C0824892123D1CA36F4D0DB24" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9630E6A6-67B0-4AF0-864F-6124807425B2}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="raw" sheetId="1" r:id="rId1"/>
     <sheet name="summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -74,8 +93,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,13 +157,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -182,7 +209,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -216,6 +243,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -250,9 +278,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -425,11 +454,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -455,9 +490,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B2">
         <v>8</v>
@@ -481,21 +516,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B3">
         <v>8</v>
       </c>
       <c r="C3">
-        <v>0.4051</v>
+        <v>0.40510000000000002</v>
       </c>
       <c r="D3">
         <v>0.2278</v>
       </c>
       <c r="E3">
-        <v>2.289940828402367</v>
+        <v>2.2899408284023668</v>
       </c>
       <c r="F3">
         <v>10</v>
@@ -507,15 +542,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B4">
         <v>8</v>
       </c>
       <c r="C4">
-        <v>0.8481</v>
+        <v>0.84809999999999997</v>
       </c>
       <c r="D4">
         <v>0.1139</v>
@@ -533,21 +568,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B5">
         <v>8</v>
       </c>
       <c r="C5">
-        <v>0.6962</v>
+        <v>0.69620000000000004</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1.593406593406593</v>
+        <v>1.5934065934065931</v>
       </c>
       <c r="F5">
         <v>10</v>
@@ -559,15 +594,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B6">
         <v>8</v>
       </c>
       <c r="C6">
-        <v>0.4937</v>
+        <v>0.49370000000000003</v>
       </c>
       <c r="D6">
         <v>0.1139</v>
@@ -585,21 +620,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B7">
         <v>8</v>
       </c>
       <c r="C7">
-        <v>0.4684</v>
+        <v>0.46839999999999998</v>
       </c>
       <c r="D7">
-        <v>0.2025</v>
+        <v>0.20250000000000001</v>
       </c>
       <c r="E7">
-        <v>2.069444444444445</v>
+        <v>2.0694444444444451</v>
       </c>
       <c r="F7">
         <v>10</v>
@@ -611,18 +646,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B8">
         <v>8</v>
       </c>
       <c r="C8">
-        <v>0.4557</v>
+        <v>0.45569999999999999</v>
       </c>
       <c r="D8">
-        <v>0.1519</v>
+        <v>0.15190000000000001</v>
       </c>
       <c r="E8">
         <v>2.16015625</v>
@@ -637,18 +672,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9">
-        <v>0.7215</v>
+        <v>0.72150000000000003</v>
       </c>
       <c r="D9">
-        <v>0.2405</v>
+        <v>0.24049999999999999</v>
       </c>
       <c r="E9">
         <v>2.019305019305019</v>
@@ -663,18 +698,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B10">
         <v>8</v>
       </c>
       <c r="C10">
-        <v>0.6203</v>
+        <v>0.62029999999999996</v>
       </c>
       <c r="D10">
-        <v>0.0759</v>
+        <v>7.5899999999999995E-2</v>
       </c>
       <c r="E10">
         <v>1.678756476683938</v>
@@ -688,22 +723,26 @@
       <c r="H10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
+      <c r="Q10">
+        <f>AVERAGE(C2:C11)</f>
+        <v>0.59115000000000006</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B11">
         <v>8</v>
       </c>
       <c r="C11">
-        <v>0.519</v>
+        <v>0.51900000000000002</v>
       </c>
       <c r="D11">
         <v>0.1772</v>
       </c>
       <c r="E11">
-        <v>1.509433962264151</v>
+        <v>1.5094339622641511</v>
       </c>
       <c r="F11">
         <v>10</v>
@@ -715,21 +754,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B12">
         <v>16</v>
       </c>
       <c r="C12">
-        <v>0.6709000000000001</v>
+        <v>0.67090000000000005</v>
       </c>
       <c r="D12">
         <v>0.2152</v>
       </c>
       <c r="E12">
-        <v>1.408791208791209</v>
+        <v>1.4087912087912089</v>
       </c>
       <c r="F12">
         <v>10</v>
@@ -741,21 +780,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B13">
         <v>16</v>
       </c>
       <c r="C13">
-        <v>0.519</v>
+        <v>0.51900000000000002</v>
       </c>
       <c r="D13">
-        <v>0.1519</v>
+        <v>0.15190000000000001</v>
       </c>
       <c r="E13">
-        <v>1.59047619047619</v>
+        <v>1.5904761904761899</v>
       </c>
       <c r="F13">
         <v>10</v>
@@ -767,21 +806,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B14">
         <v>16</v>
       </c>
       <c r="C14">
-        <v>0.5570000000000001</v>
+        <v>0.55700000000000005</v>
       </c>
       <c r="D14">
         <v>0.1772</v>
       </c>
       <c r="E14">
-        <v>2.203309692671395</v>
+        <v>2.2033096926713949</v>
       </c>
       <c r="F14">
         <v>10</v>
@@ -793,15 +832,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B15">
         <v>16</v>
       </c>
       <c r="C15">
-        <v>0.6329</v>
+        <v>0.63290000000000002</v>
       </c>
       <c r="D15">
         <v>0.2278</v>
@@ -819,21 +858,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B16">
         <v>16</v>
       </c>
       <c r="C16">
-        <v>0.8228</v>
+        <v>0.82279999999999998</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>2.197149643705463</v>
+        <v>2.1971496437054632</v>
       </c>
       <c r="F16">
         <v>10</v>
@@ -845,21 +884,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B17">
         <v>16</v>
       </c>
       <c r="C17">
-        <v>0.6582</v>
+        <v>0.65820000000000001</v>
       </c>
       <c r="D17">
-        <v>0.2025</v>
+        <v>0.20250000000000001</v>
       </c>
       <c r="E17">
-        <v>1.827014218009479</v>
+        <v>1.8270142180094791</v>
       </c>
       <c r="F17">
         <v>10</v>
@@ -871,15 +910,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B18">
         <v>16</v>
       </c>
       <c r="C18">
-        <v>0.5316</v>
+        <v>0.53159999999999996</v>
       </c>
       <c r="D18">
         <v>0.1646</v>
@@ -897,21 +936,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B19">
         <v>16</v>
       </c>
       <c r="C19">
-        <v>0.7342</v>
+        <v>0.73419999999999996</v>
       </c>
       <c r="D19">
-        <v>0.1392</v>
+        <v>0.13919999999999999</v>
       </c>
       <c r="E19">
-        <v>1.930787589498807</v>
+        <v>1.9307875894988069</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -923,9 +962,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B20">
         <v>16</v>
@@ -934,10 +973,10 @@
         <v>0.6835</v>
       </c>
       <c r="D20">
-        <v>0.1899</v>
+        <v>0.18990000000000001</v>
       </c>
       <c r="E20">
-        <v>1.533190578158458</v>
+        <v>1.5331905781584581</v>
       </c>
       <c r="F20">
         <v>10</v>
@@ -949,15 +988,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B21">
         <v>16</v>
       </c>
       <c r="C21">
-        <v>0.5063</v>
+        <v>0.50629999999999997</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -975,7 +1014,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.125</v>
       </c>
@@ -983,7 +1022,7 @@
         <v>32</v>
       </c>
       <c r="C22">
-        <v>0.5570000000000001</v>
+        <v>0.55700000000000005</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -1001,7 +1040,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.125</v>
       </c>
@@ -1009,7 +1048,7 @@
         <v>32</v>
       </c>
       <c r="C23">
-        <v>0.6456</v>
+        <v>0.64559999999999995</v>
       </c>
       <c r="D23">
         <v>0.1139</v>
@@ -1027,7 +1066,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.125</v>
       </c>
@@ -1035,7 +1074,7 @@
         <v>32</v>
       </c>
       <c r="C24">
-        <v>0.5316</v>
+        <v>0.53159999999999996</v>
       </c>
       <c r="D24">
         <v>0.1139</v>
@@ -1053,7 +1092,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.125</v>
       </c>
@@ -1061,13 +1100,13 @@
         <v>32</v>
       </c>
       <c r="C25">
-        <v>0.5823</v>
+        <v>0.58230000000000004</v>
       </c>
       <c r="D25">
-        <v>0.1266</v>
+        <v>0.12659999999999999</v>
       </c>
       <c r="E25">
-        <v>2.252747252747253</v>
+        <v>2.2527472527472532</v>
       </c>
       <c r="F25">
         <v>10</v>
@@ -1079,7 +1118,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>0.125</v>
       </c>
@@ -1087,10 +1126,10 @@
         <v>32</v>
       </c>
       <c r="C26">
-        <v>0.5949</v>
+        <v>0.59489999999999998</v>
       </c>
       <c r="D26">
-        <v>0.1519</v>
+        <v>0.15190000000000001</v>
       </c>
       <c r="E26">
         <v>1.397590361445783</v>
@@ -1105,7 +1144,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>0.125</v>
       </c>
@@ -1113,13 +1152,13 @@
         <v>32</v>
       </c>
       <c r="C27">
-        <v>0.519</v>
+        <v>0.51900000000000002</v>
       </c>
       <c r="D27">
-        <v>0.0506</v>
+        <v>5.0599999999999999E-2</v>
       </c>
       <c r="E27">
-        <v>1.730458221024259</v>
+        <v>1.7304582210242589</v>
       </c>
       <c r="F27">
         <v>10</v>
@@ -1131,7 +1170,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>0.125</v>
       </c>
@@ -1139,13 +1178,13 @@
         <v>32</v>
       </c>
       <c r="C28">
-        <v>0.5949</v>
+        <v>0.59489999999999998</v>
       </c>
       <c r="D28">
-        <v>0.1266</v>
+        <v>0.12659999999999999</v>
       </c>
       <c r="E28">
-        <v>2.298982188295165</v>
+        <v>2.2989821882951649</v>
       </c>
       <c r="F28">
         <v>10</v>
@@ -1157,7 +1196,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>0.125</v>
       </c>
@@ -1165,13 +1204,13 @@
         <v>32</v>
       </c>
       <c r="C29">
-        <v>0.6709000000000001</v>
+        <v>0.67090000000000005</v>
       </c>
       <c r="D29">
-        <v>0.1266</v>
+        <v>0.12659999999999999</v>
       </c>
       <c r="E29">
-        <v>1.569193742478941</v>
+        <v>1.5691937424789411</v>
       </c>
       <c r="F29">
         <v>10</v>
@@ -1183,7 +1222,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>0.125</v>
       </c>
@@ -1191,10 +1230,10 @@
         <v>32</v>
       </c>
       <c r="C30">
-        <v>0.6456</v>
+        <v>0.64559999999999995</v>
       </c>
       <c r="D30">
-        <v>0.0633</v>
+        <v>6.3299999999999995E-2</v>
       </c>
       <c r="E30">
         <v>1.48406862745098</v>
@@ -1209,7 +1248,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>0.125</v>
       </c>
@@ -1217,13 +1256,13 @@
         <v>32</v>
       </c>
       <c r="C31">
-        <v>0.5316</v>
+        <v>0.53159999999999996</v>
       </c>
       <c r="D31">
-        <v>0.0759</v>
+        <v>7.5899999999999995E-2</v>
       </c>
       <c r="E31">
-        <v>1.897818599311137</v>
+        <v>1.8978185993111369</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -1235,7 +1274,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>0.25</v>
       </c>
@@ -1243,13 +1282,13 @@
         <v>64</v>
       </c>
       <c r="C32">
-        <v>0.7215</v>
+        <v>0.72150000000000003</v>
       </c>
       <c r="D32">
-        <v>0.0253</v>
+        <v>2.53E-2</v>
       </c>
       <c r="E32">
-        <v>2.102346805736636</v>
+        <v>2.1023468057366359</v>
       </c>
       <c r="F32">
         <v>10</v>
@@ -1261,7 +1300,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>0.25</v>
       </c>
@@ -1269,10 +1308,10 @@
         <v>64</v>
       </c>
       <c r="C33">
-        <v>0.7089</v>
+        <v>0.70889999999999997</v>
       </c>
       <c r="D33">
-        <v>0.0633</v>
+        <v>6.3299999999999995E-2</v>
       </c>
       <c r="E33">
         <v>1.778761061946903</v>
@@ -1287,7 +1326,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>0.25</v>
       </c>
@@ -1295,13 +1334,13 @@
         <v>64</v>
       </c>
       <c r="C34">
-        <v>0.7468</v>
+        <v>0.74680000000000002</v>
       </c>
       <c r="D34">
-        <v>0.0886</v>
+        <v>8.8599999999999998E-2</v>
       </c>
       <c r="E34">
-        <v>2.375069252077562</v>
+        <v>2.3750692520775618</v>
       </c>
       <c r="F34">
         <v>10</v>
@@ -1313,7 +1352,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>0.25</v>
       </c>
@@ -1321,7 +1360,7 @@
         <v>64</v>
       </c>
       <c r="C35">
-        <v>0.5823</v>
+        <v>0.58230000000000004</v>
       </c>
       <c r="D35">
         <v>0.1139</v>
@@ -1339,7 +1378,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>0.25</v>
       </c>
@@ -1347,13 +1386,13 @@
         <v>64</v>
       </c>
       <c r="C36">
-        <v>0.6329</v>
+        <v>0.63290000000000002</v>
       </c>
       <c r="D36">
-        <v>0.0886</v>
+        <v>8.8599999999999998E-2</v>
       </c>
       <c r="E36">
-        <v>1.83943661971831</v>
+        <v>1.8394366197183101</v>
       </c>
       <c r="F36">
         <v>10</v>
@@ -1365,7 +1404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>0.25</v>
       </c>
@@ -1373,10 +1412,10 @@
         <v>64</v>
       </c>
       <c r="C37">
-        <v>0.7975</v>
+        <v>0.79749999999999999</v>
       </c>
       <c r="D37">
-        <v>0.0759</v>
+        <v>7.5899999999999995E-2</v>
       </c>
       <c r="E37">
         <v>2.282740094022834</v>
@@ -1391,7 +1430,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>0.25</v>
       </c>
@@ -1399,13 +1438,13 @@
         <v>64</v>
       </c>
       <c r="C38">
-        <v>0.7342</v>
+        <v>0.73419999999999996</v>
       </c>
       <c r="D38">
-        <v>0.1392</v>
+        <v>0.13919999999999999</v>
       </c>
       <c r="E38">
-        <v>2.164138678223185</v>
+        <v>2.1641386782231851</v>
       </c>
       <c r="F38">
         <v>10</v>
@@ -1417,7 +1456,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>0.25</v>
       </c>
@@ -1425,13 +1464,13 @@
         <v>64</v>
       </c>
       <c r="C39">
-        <v>0.7215</v>
+        <v>0.72150000000000003</v>
       </c>
       <c r="D39">
         <v>0.1139</v>
       </c>
       <c r="E39">
-        <v>2.179710144927536</v>
+        <v>2.1797101449275358</v>
       </c>
       <c r="F39">
         <v>10</v>
@@ -1443,7 +1482,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>0.25</v>
       </c>
@@ -1451,7 +1490,7 @@
         <v>64</v>
       </c>
       <c r="C40">
-        <v>0.6456</v>
+        <v>0.64559999999999995</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -1469,7 +1508,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>0.25</v>
       </c>
@@ -1477,13 +1516,13 @@
         <v>64</v>
       </c>
       <c r="C41">
-        <v>0.7975</v>
+        <v>0.79749999999999999</v>
       </c>
       <c r="D41">
-        <v>0.0506</v>
+        <v>5.0599999999999999E-2</v>
       </c>
       <c r="E41">
-        <v>1.714792899408284</v>
+        <v>1.7147928994082839</v>
       </c>
       <c r="F41">
         <v>10</v>
@@ -1495,7 +1534,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>0.5</v>
       </c>
@@ -1503,13 +1542,13 @@
         <v>128</v>
       </c>
       <c r="C42">
-        <v>0.8101</v>
+        <v>0.81010000000000004</v>
       </c>
       <c r="D42">
-        <v>0.0759</v>
+        <v>7.5899999999999995E-2</v>
       </c>
       <c r="E42">
-        <v>1.688433382137628</v>
+        <v>1.6884333821376281</v>
       </c>
       <c r="F42">
         <v>10</v>
@@ -1521,7 +1560,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>0.5</v>
       </c>
@@ -1529,13 +1568,13 @@
         <v>128</v>
       </c>
       <c r="C43">
-        <v>0.6709000000000001</v>
+        <v>0.67090000000000005</v>
       </c>
       <c r="D43">
         <v>0</v>
       </c>
       <c r="E43">
-        <v>1.889842632331903</v>
+        <v>1.8898426323319031</v>
       </c>
       <c r="F43">
         <v>10</v>
@@ -1547,7 +1586,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>0.5</v>
       </c>
@@ -1555,10 +1594,10 @@
         <v>128</v>
       </c>
       <c r="C44">
-        <v>0.7089</v>
+        <v>0.70889999999999997</v>
       </c>
       <c r="D44">
-        <v>0.0506</v>
+        <v>5.0599999999999999E-2</v>
       </c>
       <c r="E44">
         <v>1.426530612244898</v>
@@ -1573,7 +1612,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>0.5</v>
       </c>
@@ -1581,7 +1620,7 @@
         <v>128</v>
       </c>
       <c r="C45">
-        <v>0.6582</v>
+        <v>0.65820000000000001</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -1599,7 +1638,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>0.5</v>
       </c>
@@ -1607,10 +1646,10 @@
         <v>128</v>
       </c>
       <c r="C46">
-        <v>0.6709000000000001</v>
+        <v>0.67090000000000005</v>
       </c>
       <c r="D46">
-        <v>0.0506</v>
+        <v>5.0599999999999999E-2</v>
       </c>
       <c r="E46">
         <v>1.826073232323232</v>
@@ -1625,7 +1664,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>0.5</v>
       </c>
@@ -1633,13 +1672,13 @@
         <v>128</v>
       </c>
       <c r="C47">
-        <v>0.7595</v>
+        <v>0.75949999999999995</v>
       </c>
       <c r="D47">
-        <v>0.0253</v>
+        <v>2.53E-2</v>
       </c>
       <c r="E47">
-        <v>1.943856554967666</v>
+        <v>1.9438565549676661</v>
       </c>
       <c r="F47">
         <v>10</v>
@@ -1651,7 +1690,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>0.5</v>
       </c>
@@ -1662,10 +1701,10 @@
         <v>0.6835</v>
       </c>
       <c r="D48">
-        <v>0.0759</v>
+        <v>7.5899999999999995E-2</v>
       </c>
       <c r="E48">
-        <v>1.441436138905238</v>
+        <v>1.4414361389052379</v>
       </c>
       <c r="F48">
         <v>10</v>
@@ -1677,7 +1716,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>0.5</v>
       </c>
@@ -1685,10 +1724,10 @@
         <v>128</v>
       </c>
       <c r="C49">
-        <v>0.7215</v>
+        <v>0.72150000000000003</v>
       </c>
       <c r="D49">
-        <v>0.0506</v>
+        <v>5.0599999999999999E-2</v>
       </c>
       <c r="E49">
         <v>1.478494623655914</v>
@@ -1703,7 +1742,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>0.5</v>
       </c>
@@ -1711,13 +1750,13 @@
         <v>128</v>
       </c>
       <c r="C50">
-        <v>0.6962</v>
+        <v>0.69620000000000004</v>
       </c>
       <c r="D50">
         <v>0</v>
       </c>
       <c r="E50">
-        <v>1.832644628099174</v>
+        <v>1.8326446280991739</v>
       </c>
       <c r="F50">
         <v>10</v>
@@ -1729,7 +1768,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>0.5</v>
       </c>
@@ -1740,10 +1779,10 @@
         <v>0.7722</v>
       </c>
       <c r="D51">
-        <v>0.0633</v>
+        <v>6.3299999999999995E-2</v>
       </c>
       <c r="E51">
-        <v>1.980030721966206</v>
+        <v>1.9800307219662061</v>
       </c>
       <c r="F51">
         <v>10</v>
@@ -1761,11 +1800,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1809,39 +1859,39 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B2">
         <v>8</v>
       </c>
       <c r="C2">
-        <v>0.5911500000000001</v>
+        <v>0.59115000000000006</v>
       </c>
       <c r="D2">
-        <v>0.4051</v>
+        <v>0.40510000000000002</v>
       </c>
       <c r="E2">
-        <v>0.8481</v>
+        <v>0.84809999999999997</v>
       </c>
       <c r="F2">
-        <v>0.5911500000000001</v>
+        <v>0.59115000000000006</v>
       </c>
       <c r="G2">
-        <v>0.4051</v>
+        <v>0.40510000000000002</v>
       </c>
       <c r="H2">
-        <v>0.8481</v>
+        <v>0.84809999999999997</v>
       </c>
       <c r="I2">
-        <v>1.889790836323891</v>
+        <v>1.8897908363238911</v>
       </c>
       <c r="J2">
-        <v>1.509433962264151</v>
+        <v>1.5094339622641511</v>
       </c>
       <c r="K2">
-        <v>2.289940828402367</v>
+        <v>2.2899408284023668</v>
       </c>
       <c r="L2">
         <v>10</v>
@@ -1853,36 +1903,36 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B3">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>0.63164</v>
+        <v>0.63163999999999998</v>
       </c>
       <c r="D3">
-        <v>0.5063</v>
+        <v>0.50629999999999997</v>
       </c>
       <c r="E3">
-        <v>0.8228</v>
+        <v>0.82279999999999998</v>
       </c>
       <c r="F3">
-        <v>0.63164</v>
+        <v>0.63163999999999998</v>
       </c>
       <c r="G3">
-        <v>0.5063</v>
+        <v>0.50629999999999997</v>
       </c>
       <c r="H3">
-        <v>0.8228</v>
+        <v>0.82279999999999998</v>
       </c>
       <c r="I3">
-        <v>1.818517073479552</v>
+        <v>1.8185170734795519</v>
       </c>
       <c r="J3">
-        <v>1.408791208791209</v>
+        <v>1.4087912087912089</v>
       </c>
       <c r="K3">
         <v>2.371359223300971</v>
@@ -1897,7 +1947,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0.125</v>
       </c>
@@ -1905,22 +1955,22 @@
         <v>32</v>
       </c>
       <c r="C4">
-        <v>0.58734</v>
+        <v>0.58733999999999997</v>
       </c>
       <c r="D4">
-        <v>0.519</v>
+        <v>0.51900000000000002</v>
       </c>
       <c r="E4">
-        <v>0.6709000000000001</v>
+        <v>0.67090000000000005</v>
       </c>
       <c r="F4">
-        <v>0.58734</v>
+        <v>0.58733999999999997</v>
       </c>
       <c r="G4">
-        <v>0.519</v>
+        <v>0.51900000000000002</v>
       </c>
       <c r="H4">
-        <v>0.6709000000000001</v>
+        <v>0.67090000000000005</v>
       </c>
       <c r="I4">
         <v>1.720352629178078</v>
@@ -1929,7 +1979,7 @@
         <v>1.341379310344827</v>
       </c>
       <c r="K4">
-        <v>2.298982188295165</v>
+        <v>2.2989821882951649</v>
       </c>
       <c r="L4">
         <v>10</v>
@@ -1941,7 +1991,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>0.25</v>
       </c>
@@ -1952,19 +2002,19 @@
         <v>0.70887</v>
       </c>
       <c r="D5">
-        <v>0.5823</v>
+        <v>0.58230000000000004</v>
       </c>
       <c r="E5">
-        <v>0.7975</v>
+        <v>0.79749999999999999</v>
       </c>
       <c r="F5">
         <v>0.70887</v>
       </c>
       <c r="G5">
-        <v>0.5823</v>
+        <v>0.58230000000000004</v>
       </c>
       <c r="H5">
-        <v>0.7975</v>
+        <v>0.79749999999999999</v>
       </c>
       <c r="I5">
         <v>1.984516790452644</v>
@@ -1973,7 +2023,7 @@
         <v>1.558425584255843</v>
       </c>
       <c r="K5">
-        <v>2.375069252077562</v>
+        <v>2.3750692520775618</v>
       </c>
       <c r="L5">
         <v>10</v>
@@ -1985,7 +2035,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.5</v>
       </c>
@@ -1993,31 +2043,31 @@
         <v>128</v>
       </c>
       <c r="C6">
-        <v>0.71519</v>
+        <v>0.71518999999999999</v>
       </c>
       <c r="D6">
-        <v>0.6582</v>
+        <v>0.65820000000000001</v>
       </c>
       <c r="E6">
-        <v>0.8101</v>
+        <v>0.81010000000000004</v>
       </c>
       <c r="F6">
-        <v>0.71519</v>
+        <v>0.71518999999999999</v>
       </c>
       <c r="G6">
-        <v>0.6582</v>
+        <v>0.65820000000000001</v>
       </c>
       <c r="H6">
-        <v>0.8101</v>
+        <v>0.81010000000000004</v>
       </c>
       <c r="I6">
-        <v>1.728815612711759</v>
+        <v>1.7288156127117591</v>
       </c>
       <c r="J6">
         <v>1.426530612244898</v>
       </c>
       <c r="K6">
-        <v>1.980030721966206</v>
+        <v>1.9800307219662061</v>
       </c>
       <c r="L6">
         <v>10</v>

</xml_diff>